<commit_message>
Update BPP codebase with HF tasks, batch runners, and safe API key placeholders.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/logs/codenames_collaborative/gpt-3.5-turbo_wo_sys_mes/accuracy_results_gpt35-turbo_wo_sys_mes.xlsx
+++ b/logs/codenames_collaborative/gpt-3.5-turbo_wo_sys_mes/accuracy_results_gpt35-turbo_wo_sys_mes.xlsx
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -481,7 +481,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -504,7 +504,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -550,7 +550,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -573,7 +573,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -596,7 +596,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -642,7 +642,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -665,7 +665,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -688,7 +688,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -711,7 +711,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -734,7 +734,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -757,7 +757,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -780,7 +780,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -803,7 +803,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -826,7 +826,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -849,7 +849,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -872,7 +872,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -895,7 +895,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -918,7 +918,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -941,7 +941,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -964,7 +964,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -987,7 +987,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1010,7 +1010,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1033,7 +1033,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1056,7 +1056,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1079,7 +1079,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1102,7 +1102,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1125,7 +1125,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1148,7 +1148,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1171,7 +1171,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1194,7 +1194,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1217,7 +1217,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1240,7 +1240,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1263,7 +1263,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1286,7 +1286,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1309,7 +1309,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1332,7 +1332,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1355,7 +1355,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1378,7 +1378,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1401,7 +1401,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1424,7 +1424,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1447,7 +1447,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1470,7 +1470,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1493,7 +1493,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1516,7 +1516,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1539,7 +1539,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1562,7 +1562,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1585,7 +1585,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1608,7 +1608,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1633,7 +1633,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1656,7 +1656,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1679,7 +1679,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1702,7 +1702,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1725,7 +1725,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1748,7 +1748,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1771,7 +1771,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1794,7 +1794,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1817,7 +1817,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1840,7 +1840,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1863,7 +1863,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1886,7 +1886,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1909,7 +1909,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1932,7 +1932,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1955,7 +1955,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1978,7 +1978,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2001,7 +2001,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2024,7 +2024,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2047,7 +2047,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2070,7 +2070,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2093,7 +2093,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2116,7 +2116,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2139,7 +2139,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2162,7 +2162,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2185,7 +2185,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2208,7 +2208,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2231,7 +2231,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2254,7 +2254,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2277,7 +2277,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2300,7 +2300,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2323,7 +2323,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2346,7 +2346,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2369,7 +2369,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2392,7 +2392,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2415,7 +2415,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2438,7 +2438,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2461,7 +2461,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2484,7 +2484,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2530,7 +2530,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2553,7 +2553,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2576,7 +2576,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2599,7 +2599,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2622,7 +2622,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2645,7 +2645,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2668,7 +2668,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2691,7 +2691,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2714,7 +2714,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2737,7 +2737,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2760,7 +2760,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2783,7 +2783,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-macro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2808,7 +2808,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2831,7 +2831,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2854,7 +2854,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2877,7 +2877,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2900,7 +2900,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2923,7 +2923,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -2946,7 +2946,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -2969,7 +2969,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2992,7 +2992,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3015,7 +3015,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -3038,7 +3038,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3061,7 +3061,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3084,7 +3084,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3130,7 +3130,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3153,7 +3153,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3176,7 +3176,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3199,7 +3199,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3222,7 +3222,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3245,7 +3245,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3268,7 +3268,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3291,7 +3291,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3314,7 +3314,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3337,7 +3337,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3360,7 +3360,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3383,7 +3383,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3406,7 +3406,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3429,7 +3429,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3452,7 +3452,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3475,7 +3475,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3498,7 +3498,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -3521,7 +3521,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3544,7 +3544,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3567,7 +3567,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3590,7 +3590,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3613,7 +3613,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3636,7 +3636,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3659,7 +3659,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -3682,7 +3682,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3705,7 +3705,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3728,7 +3728,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3751,7 +3751,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3774,7 +3774,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3797,7 +3797,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -3820,7 +3820,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -3843,7 +3843,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -3889,7 +3889,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -3912,7 +3912,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -3935,7 +3935,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -3958,7 +3958,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-meso_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -3983,7 +3983,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4006,7 +4006,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -4029,7 +4029,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4052,7 +4052,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4075,7 +4075,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4098,7 +4098,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4121,7 +4121,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4144,7 +4144,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4167,7 +4167,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4190,7 +4190,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -4213,7 +4213,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -4236,7 +4236,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4259,7 +4259,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4282,7 +4282,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4305,7 +4305,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -4328,7 +4328,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -4351,7 +4351,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -4374,7 +4374,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4397,7 +4397,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4420,7 +4420,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4443,7 +4443,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4466,7 +4466,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4489,7 +4489,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -4512,7 +4512,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4535,7 +4535,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4558,7 +4558,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4581,7 +4581,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4604,7 +4604,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -4627,7 +4627,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4650,7 +4650,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -4673,7 +4673,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4696,7 +4696,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4719,7 +4719,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -4742,7 +4742,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -4765,7 +4765,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -4788,7 +4788,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -4811,7 +4811,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -4834,7 +4834,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -4857,7 +4857,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -4880,7 +4880,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -4903,7 +4903,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -4926,7 +4926,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -4949,7 +4949,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -4972,7 +4972,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -4995,7 +4995,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5018,7 +5018,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5041,7 +5041,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5064,7 +5064,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5110,7 +5110,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -5133,7 +5133,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-micro_bpp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5158,7 +5158,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5181,7 +5181,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5204,7 +5204,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5227,7 +5227,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5250,7 +5250,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5273,7 +5273,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5296,7 +5296,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5319,7 +5319,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5342,7 +5342,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5365,7 +5365,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5388,7 +5388,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5411,7 +5411,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5434,7 +5434,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5457,7 +5457,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -5480,7 +5480,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -5503,7 +5503,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -5526,7 +5526,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5549,7 +5549,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5572,7 +5572,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -5595,7 +5595,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -5618,7 +5618,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5641,7 +5641,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -5664,7 +5664,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -5710,7 +5710,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -5733,7 +5733,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -5756,7 +5756,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -5779,7 +5779,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -5802,7 +5802,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -5825,7 +5825,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -5848,7 +5848,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -5871,7 +5871,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -5894,7 +5894,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -5917,7 +5917,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -5940,7 +5940,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -5963,7 +5963,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -5986,7 +5986,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -6009,7 +6009,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -6032,7 +6032,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6055,7 +6055,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6078,7 +6078,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6101,7 +6101,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -6124,7 +6124,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -6147,7 +6147,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -6170,7 +6170,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -6193,7 +6193,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -6216,7 +6216,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -6239,7 +6239,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -6262,7 +6262,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6285,7 +6285,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6308,7 +6308,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-spp_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6333,7 +6333,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -6356,7 +6356,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -6379,7 +6379,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -6402,7 +6402,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -6425,7 +6425,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -6448,7 +6448,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6471,7 +6471,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -6494,7 +6494,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6517,7 +6517,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -6540,7 +6540,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6563,7 +6563,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -6586,7 +6586,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -6609,7 +6609,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -6632,7 +6632,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -6655,7 +6655,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -6678,7 +6678,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -6701,7 +6701,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -6724,7 +6724,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -6747,7 +6747,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -6770,7 +6770,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -6793,7 +6793,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
@@ -6816,7 +6816,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -6839,7 +6839,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -6862,7 +6862,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -6885,7 +6885,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -6908,7 +6908,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -6931,7 +6931,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -6954,7 +6954,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -6977,7 +6977,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -7000,7 +7000,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -7023,7 +7023,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -7046,7 +7046,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7069,7 +7069,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7092,7 +7092,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -7115,7 +7115,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -7138,7 +7138,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7161,7 +7161,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7184,7 +7184,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7207,7 +7207,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7230,7 +7230,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -7253,7 +7253,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
@@ -7276,7 +7276,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
@@ -7299,7 +7299,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -7322,7 +7322,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -7345,7 +7345,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -7368,7 +7368,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
@@ -7391,7 +7391,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -7414,7 +7414,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
@@ -7437,7 +7437,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7460,7 +7460,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7483,7 +7483,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50__wo_sys.jsonl</t>
+          <t>codenames_50.jsonl__method-standard_model-gpt-3.5-turbo_temp-_temp-0.0_topp-_topp-1.0_start0-end50_run01__wo_sys.jsonl</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">

</xml_diff>